<commit_message>
rush series 3: lineups, 37 mapas, chave de dupla eliminacao e pontos
- inscricao do Challengermode cadastrada: 33 jogadores novos (Milanga pelo
  PUUID do JSON), 15 nicks novos e Parzival como puuid 2 do Kaizin
- equipes novas: UFRN Tirana, UFU Saints Onyx e Incinera E-Sports (Carcaras,
  Trigons e Virtus perdem os jogadores e ficam inativas), Azure Bears Spotline
  e Polaris; amistoso sem elenco, so com completes: FEI Last Dance, FEI Capim,
  MackLogic Wine e Atletica Sustenta
- 37 de 38 mapas no acervo; a P2 nao existe na Riot; W.O. nas P20, P43, P49
  e P52
- override com chave de 32 vagas, pontos 35/30/25/20/15/10/5/0/0 e fase final
  na serie 62
- logos e cores das equipes novas; round_state_winrates recalculado
- ranking de 20/10: CEUB Vulgaris 18 -> 11, MackLogic White entra em 24 e
  INATEL Gray em 50

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados_excel/players.xlsx
+++ b/dados_excel/players.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P711"/>
+  <dimension ref="A1:Q744"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="24" defaultRowHeight="14.4"/>
   <cols>
     <col width="15.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -563,6 +563,11 @@
           <t>nick 5</t>
         </is>
       </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>team 6</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3723,9 +3728,14 @@
           <t>ufu_saints</t>
         </is>
       </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>ufu_saints_onyx</t>
+        </is>
+      </c>
       <c r="G111" t="inlineStr">
         <is>
-          <t>ufu_saints</t>
+          <t>ufu_saints_onyx</t>
         </is>
       </c>
       <c r="I111" t="inlineStr">
@@ -3937,9 +3947,14 @@
           <t>ufu_saints_trigons</t>
         </is>
       </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>ufu_saints_onyx</t>
+        </is>
+      </c>
       <c r="G118" t="inlineStr">
         <is>
-          <t>ufu_saints_trigons</t>
+          <t>ufu_saints_onyx</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -3950,6 +3965,11 @@
       <c r="L118" t="inlineStr">
         <is>
           <t>warplane#gsN</t>
+        </is>
+      </c>
+      <c r="M118" t="inlineStr">
+        <is>
+          <t>gsN#TASR</t>
         </is>
       </c>
     </row>
@@ -4006,6 +4026,11 @@
           <t>lopes cabral 13#sidny</t>
         </is>
       </c>
+      <c r="M120" t="inlineStr">
+        <is>
+          <t>Houndoom#lmx</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4347,9 +4372,14 @@
           <t>ufrn_carcaras</t>
         </is>
       </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>ufrn_tirana</t>
+        </is>
+      </c>
       <c r="G133" t="inlineStr">
         <is>
-          <t>ufrn_carcaras</t>
+          <t>ufrn_tirana</t>
         </is>
       </c>
       <c r="I133" t="inlineStr">
@@ -4360,6 +4390,11 @@
       <c r="L133" t="inlineStr">
         <is>
           <t>gbr is back#lindo</t>
+        </is>
+      </c>
+      <c r="M133" t="inlineStr">
+        <is>
+          <t>jung#hans</t>
         </is>
       </c>
     </row>
@@ -4374,9 +4409,14 @@
           <t>ufrn_carcaras</t>
         </is>
       </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>ufrn_tirana</t>
+        </is>
+      </c>
       <c r="G134" t="inlineStr">
         <is>
-          <t>ufrn_carcaras</t>
+          <t>ufrn_tirana</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -4428,9 +4468,14 @@
           <t>ufrn_carcaras</t>
         </is>
       </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>ufrn_tirana</t>
+        </is>
+      </c>
       <c r="G136" t="inlineStr">
         <is>
-          <t>ufrn_carcaras</t>
+          <t>ufrn_tirana</t>
         </is>
       </c>
       <c r="I136" t="inlineStr">
@@ -4455,9 +4500,14 @@
           <t>ufrn_carcaras</t>
         </is>
       </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>ufrn_tirana</t>
+        </is>
+      </c>
       <c r="G137" t="inlineStr">
         <is>
-          <t>ufrn_carcaras</t>
+          <t>ufrn_tirana</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -4465,9 +4515,19 @@
           <t>DgjD8cHoPEUZe3LH6OvWCbS8c5mmcEdrDzWbMpFaM9e5JIv_i90Hf4YLULdo7gDA5tYfRMzmV5neZA</t>
         </is>
       </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>x3-xgAqsNfekgbOnRbwkErykZOKVAP7pgy4jfQDSNXKavyQ6344ZOeXl18vOhxFcTvPMCIUuwW_sDQ</t>
+        </is>
+      </c>
       <c r="L137" t="inlineStr">
         <is>
           <t>oKaizin#Sett</t>
+        </is>
+      </c>
+      <c r="M137" t="inlineStr">
+        <is>
+          <t>Parzival#IWNL</t>
         </is>
       </c>
     </row>
@@ -4529,6 +4589,11 @@
           <t>BBL lovers rock#1912</t>
         </is>
       </c>
+      <c r="N139" t="inlineStr">
+        <is>
+          <t>berna#1912</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -4632,9 +4697,14 @@
           <t>minerva_artemis</t>
         </is>
       </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>ufrj_minerva</t>
+        </is>
+      </c>
       <c r="G143" t="inlineStr">
         <is>
-          <t>minerva_artemis</t>
+          <t>ufrj_minerva</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -4939,9 +5009,14 @@
           <t>ufpe_virtus</t>
         </is>
       </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>incinera_esports</t>
+        </is>
+      </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>ufpe_virtus</t>
+          <t>incinera_esports</t>
         </is>
       </c>
       <c r="I154" t="inlineStr">
@@ -4966,9 +5041,14 @@
           <t>ufpe_virtus</t>
         </is>
       </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>incinera_esports</t>
+        </is>
+      </c>
       <c r="G155" t="inlineStr">
         <is>
-          <t>ufpe_virtus</t>
+          <t>incinera_esports</t>
         </is>
       </c>
       <c r="I155" t="inlineStr">
@@ -4993,9 +5073,14 @@
           <t>ufpe_virtus</t>
         </is>
       </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>incinera_esports</t>
+        </is>
+      </c>
       <c r="G156" t="inlineStr">
         <is>
-          <t>ufpe_virtus</t>
+          <t>incinera_esports</t>
         </is>
       </c>
       <c r="I156" t="inlineStr">
@@ -9688,7 +9773,7 @@
       </c>
       <c r="H320" t="inlineStr">
         <is>
-          <t>macklogic_red</t>
+          <t>macklogic_red; macklogic_wine</t>
         </is>
       </c>
       <c r="I320" t="inlineStr">
@@ -9699,6 +9784,11 @@
       <c r="L320" t="inlineStr">
         <is>
           <t>LOGIC gabs#lolô</t>
+        </is>
+      </c>
+      <c r="M320" t="inlineStr">
+        <is>
+          <t>LGC gabs cu1ud0#lolo</t>
         </is>
       </c>
     </row>
@@ -9807,6 +9897,11 @@
           <t>macklogic_red</t>
         </is>
       </c>
+      <c r="H323" t="inlineStr">
+        <is>
+          <t>macklogic_wine</t>
+        </is>
+      </c>
       <c r="I323" t="inlineStr">
         <is>
           <t>rFEJgUoul02DPJmUvpEPZlGn0rxTcS2zX8gQa0fm72gckzMh-5o1tmkzyzRjfufFa7mMDcRk5EhXHw</t>
@@ -10033,6 +10128,11 @@
           <t>macklogic_rainbow</t>
         </is>
       </c>
+      <c r="H331" t="inlineStr">
+        <is>
+          <t>macklogic_wine</t>
+        </is>
+      </c>
       <c r="I331" t="inlineStr">
         <is>
           <t>DpKN_eGJaVSBRddfDE72xX67drRNAKrUG42Ys9vC5nlI__06S4XLPRK0g7rwC3n4aMgmtYSg51IzeA</t>
@@ -10841,6 +10941,11 @@
           <t>INTL tambaqui#math</t>
         </is>
       </c>
+      <c r="M360" t="inlineStr">
+        <is>
+          <t>tambaqui#math</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -10873,6 +10978,11 @@
           <t>INTL chica#dan</t>
         </is>
       </c>
+      <c r="N361" t="inlineStr">
+        <is>
+          <t>Chica Moedas#nata</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -12944,6 +13054,11 @@
           <t>fei_whiteowls</t>
         </is>
       </c>
+      <c r="H434" t="inlineStr">
+        <is>
+          <t>fei_last_dance</t>
+        </is>
+      </c>
       <c r="I434" t="inlineStr">
         <is>
           <t>cvmNBm2AO5MLr0znGuB790m_Y1Sp9lpdql5US15V8wFLIZoWHBbhgCLq9q1fCq-xg4ILWJAdXahEyg</t>
@@ -12981,6 +13096,11 @@
           <t>fei_whiteowls</t>
         </is>
       </c>
+      <c r="H435" t="inlineStr">
+        <is>
+          <t>fei_capim</t>
+        </is>
+      </c>
       <c r="I435" t="inlineStr">
         <is>
           <t>EGhBQHDEXsBAc1DryXTp0v3g7E-hkkGZnFoi1_2l1Zzt4SAVUh9gR_9ZYhPu8JW5k9fegie2I-BtZg</t>
@@ -13023,6 +13143,11 @@
           <t>fei_whiteowls</t>
         </is>
       </c>
+      <c r="H436" t="inlineStr">
+        <is>
+          <t>fei_capim</t>
+        </is>
+      </c>
       <c r="I436" t="inlineStr">
         <is>
           <t>YLckYbNDIUHqyLoJeMhaECKqLC4nW4OboUi3qOo2LiwxyG6p59hYLwCbzU5HnLfXQ368G0J1C9UVkw</t>
@@ -13055,6 +13180,11 @@
           <t>fei_whiteowls</t>
         </is>
       </c>
+      <c r="H437" t="inlineStr">
+        <is>
+          <t>fei_capim</t>
+        </is>
+      </c>
       <c r="I437" t="inlineStr">
         <is>
           <t>qt7b90Pn8ZsT9ZhqHNBMLkKP574PJlUD0p0XHFmiorLv0RqiXAv64ibJFbaizJQYzztuLxQeNUyDDw</t>
@@ -13073,6 +13203,11 @@
       <c r="N437" t="inlineStr">
         <is>
           <t>Kayden#wired</t>
+        </is>
+      </c>
+      <c r="O437" t="inlineStr">
+        <is>
+          <t>azul viagra#line</t>
         </is>
       </c>
     </row>
@@ -13161,6 +13296,11 @@
           <t>fei_darkowls</t>
         </is>
       </c>
+      <c r="H440" t="inlineStr">
+        <is>
+          <t>fei_last_dance</t>
+        </is>
+      </c>
       <c r="I440" t="inlineStr">
         <is>
           <t>khFydt699IQigzJY9zSaAWVEkODol7bZwiESFtYF1eAQOpMTlLg2wrAGYYs5bXuyqac5K3fZHqh_Hg</t>
@@ -13188,6 +13328,11 @@
           <t>fei_darkowls</t>
         </is>
       </c>
+      <c r="H441" t="inlineStr">
+        <is>
+          <t>fei_last_dance</t>
+        </is>
+      </c>
       <c r="I441" t="inlineStr">
         <is>
           <t>Oay2zIMCBj4vVXFtpJubolx1gBAqX770Kj_or0iBQ_8ibrtSyrlOPCA70fKWydpigSZwSxaBTYZQpA</t>
@@ -13230,6 +13375,11 @@
           <t>fei_darkowls</t>
         </is>
       </c>
+      <c r="H442" t="inlineStr">
+        <is>
+          <t>fei_capim</t>
+        </is>
+      </c>
       <c r="I442" t="inlineStr">
         <is>
           <t>AWNQ_CNOeyRjpXJEZk3h2mEoZqU1xAAXlDiv3ilDZ249Ot4BMF--jyHQE4Jq6TQlFCjafLzD0wdD4g</t>
@@ -13277,6 +13427,11 @@
           <t>fei_darkowls</t>
         </is>
       </c>
+      <c r="H443" t="inlineStr">
+        <is>
+          <t>fei_capim</t>
+        </is>
+      </c>
       <c r="I443" t="inlineStr">
         <is>
           <t>yKOJaoTc-2NZaO7S-9nascHATOsM4Jyv1wK6fIdT7A1XNzsS-NSAFvj56O4r01rUz13UH_Rh41VWVA</t>
@@ -13827,6 +13982,11 @@
           <t>ceub_octopus_vulgaris</t>
         </is>
       </c>
+      <c r="H463" t="inlineStr">
+        <is>
+          <t>atletica_sustenta</t>
+        </is>
+      </c>
       <c r="I463" t="inlineStr">
         <is>
           <t>x2CH5wSlgIpaT7Pe44AXQb6Eb1phYUDI2a7wqfej6p0CdhqbtzCmLyCQ8KPyniuzUjnZ1ACCi87c_Q</t>
@@ -14457,7 +14617,7 @@
       </c>
       <c r="G482" t="inlineStr">
         <is>
-          <t>caap_malditos</t>
+          <t>caap_auroras</t>
         </is>
       </c>
       <c r="I482" t="inlineStr">
@@ -14473,6 +14633,11 @@
       <c r="M482" t="inlineStr">
         <is>
           <t>mist#2706</t>
+        </is>
+      </c>
+      <c r="Q482" t="inlineStr">
+        <is>
+          <t>caap_auroras</t>
         </is>
       </c>
     </row>
@@ -15435,6 +15600,11 @@
           <t>dvd isnt perfect#yas</t>
         </is>
       </c>
+      <c r="M512" t="inlineStr">
+        <is>
+          <t>dvd is smooth#clean</t>
+        </is>
+      </c>
     </row>
     <row r="513">
       <c r="A513" t="inlineStr">
@@ -15489,6 +15659,11 @@
           <t>s kd#alskd</t>
         </is>
       </c>
+      <c r="M514" t="inlineStr">
+        <is>
+          <t>s kd anti comuna#alskd</t>
+        </is>
+      </c>
     </row>
     <row r="515">
       <c r="A515" t="inlineStr">
@@ -15516,6 +15691,11 @@
           <t>Andronicca#mel</t>
         </is>
       </c>
+      <c r="M515" t="inlineStr">
+        <is>
+          <t>mel#jpb</t>
+        </is>
+      </c>
     </row>
     <row r="516">
       <c r="A516" t="inlineStr">
@@ -15954,9 +16134,14 @@
           <t>azure_bears_black</t>
         </is>
       </c>
+      <c r="E529" t="inlineStr">
+        <is>
+          <t>azure_bears_silver</t>
+        </is>
+      </c>
       <c r="G529" t="inlineStr">
         <is>
-          <t>azure_bears_black</t>
+          <t>azure_bears_silver</t>
         </is>
       </c>
       <c r="I529" t="inlineStr">
@@ -17711,9 +17896,14 @@
           <t>ceub_octopus</t>
         </is>
       </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>ceub_octopus_vulgaris</t>
+        </is>
+      </c>
       <c r="G585" t="inlineStr">
         <is>
-          <t>ceub_octopus</t>
+          <t>ceub_octopus_vulgaris</t>
         </is>
       </c>
       <c r="I585" t="inlineStr">
@@ -17854,6 +18044,11 @@
           <t>ikone#carti</t>
         </is>
       </c>
+      <c r="N589" t="inlineStr">
+        <is>
+          <t>cartunez#teenx</t>
+        </is>
+      </c>
     </row>
     <row r="590">
       <c r="A590" t="inlineStr">
@@ -17871,6 +18066,11 @@
           <t>ceub_octopus_vulgaris</t>
         </is>
       </c>
+      <c r="H590" t="inlineStr">
+        <is>
+          <t>atletica_sustenta</t>
+        </is>
+      </c>
       <c r="I590" t="inlineStr">
         <is>
           <t>TCUxMtkwuASrXI-eKQVBwhVWy64-Czu8fWw_VYLrCd_FYHVDOzXVX3QDMmrRTQVamSuYtfXR_JpHIg</t>
@@ -19303,6 +19503,11 @@
           <t>DG  叶#Deus</t>
         </is>
       </c>
+      <c r="M646" t="inlineStr">
+        <is>
+          <t>DG  神#Anjo</t>
+        </is>
+      </c>
     </row>
     <row r="647">
       <c r="A647" t="inlineStr">
@@ -19870,9 +20075,14 @@
           <t>ufu_saints_trigons</t>
         </is>
       </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>ufu_saints_onyx</t>
+        </is>
+      </c>
       <c r="G667" t="inlineStr">
         <is>
-          <t>ufu_saints_trigons</t>
+          <t>ufu_saints_onyx</t>
         </is>
       </c>
       <c r="I667" t="inlineStr">
@@ -19897,9 +20107,14 @@
           <t>ufu_saints_trigons</t>
         </is>
       </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>ufu_saints_onyx</t>
+        </is>
+      </c>
       <c r="G668" t="inlineStr">
         <is>
-          <t>ufu_saints_trigons</t>
+          <t>ufu_saints_onyx</t>
         </is>
       </c>
       <c r="I668" t="inlineStr">
@@ -19924,9 +20139,14 @@
           <t>ufu_saints_trigons</t>
         </is>
       </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>ufu_saints_onyx</t>
+        </is>
+      </c>
       <c r="G669" t="inlineStr">
         <is>
-          <t>ufu_saints_trigons</t>
+          <t>ufu_saints_onyx</t>
         </is>
       </c>
       <c r="I669" t="inlineStr">
@@ -20668,6 +20888,11 @@
           <t>Jungkook#giu</t>
         </is>
       </c>
+      <c r="M696" t="inlineStr">
+        <is>
+          <t>ruyezi#giu</t>
+        </is>
+      </c>
     </row>
     <row r="697">
       <c r="A697" t="inlineStr">
@@ -20722,6 +20947,11 @@
           <t>Elden#Rot</t>
         </is>
       </c>
+      <c r="M698" t="inlineStr">
+        <is>
+          <t>Zer00#Fear</t>
+        </is>
+      </c>
     </row>
     <row r="699">
       <c r="A699" t="inlineStr">
@@ -20793,6 +21023,11 @@
           <t>macklogic_white</t>
         </is>
       </c>
+      <c r="H701" t="inlineStr">
+        <is>
+          <t>macklogic_wine</t>
+        </is>
+      </c>
       <c r="I701" t="inlineStr">
         <is>
           <t>heDjhUTOfks5EfPbAo4f-I22sUyGjYg2YFzpV8ZgULa4VdRXy_bTWm6ChRTq5OWYxJHzdvNUiav5fg</t>
@@ -21071,6 +21306,862 @@
       <c r="L711" t="inlineStr">
         <is>
           <t>GLEP#GIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>Randon</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>ufrn_tirana</t>
+        </is>
+      </c>
+      <c r="G712" t="inlineStr">
+        <is>
+          <t>ufrn_tirana</t>
+        </is>
+      </c>
+      <c r="I712" t="inlineStr">
+        <is>
+          <t>_Ktp5rRC27VOPwOru77zfVnBpUOLuW-EmgZ11tInm3dpdwXUYdIvcH1g9-3YdZNMz6o4z2fwsdgBjw</t>
+        </is>
+      </c>
+      <c r="L712" t="inlineStr">
+        <is>
+          <t>Randon#95754</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>pipo166</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>ceub_octopus_vulgaris</t>
+        </is>
+      </c>
+      <c r="G713" t="inlineStr">
+        <is>
+          <t>ceub_octopus_vulgaris</t>
+        </is>
+      </c>
+      <c r="I713" t="inlineStr">
+        <is>
+          <t>Da_w5mHsk6pyrRKtxWkp9S5mSOzY5hUtjCGSrjuqlSoBW5XjgBz1UW5jkELqXUy2UVwyaACK415sBQ</t>
+        </is>
+      </c>
+      <c r="L713" t="inlineStr">
+        <is>
+          <t>about#soul</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>PedroBSilva</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>ufmt_turuna</t>
+        </is>
+      </c>
+      <c r="G714" t="inlineStr">
+        <is>
+          <t>ufmt_turuna</t>
+        </is>
+      </c>
+      <c r="I714" t="inlineStr">
+        <is>
+          <t>0jpTPGN_JEwYgCuTUZsxHWHaLoDBphYgcttzYsfDyFGJzehatjfpv4qkrK11olQ7tYrSD2XC7A--yw</t>
+        </is>
+      </c>
+      <c r="L714" t="inlineStr">
+        <is>
+          <t>louco de whisky#bruno</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>Arkseiro</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>azure_bears_silver</t>
+        </is>
+      </c>
+      <c r="G715" t="inlineStr">
+        <is>
+          <t>azure_bears_silver</t>
+        </is>
+      </c>
+      <c r="I715" t="inlineStr">
+        <is>
+          <t>0lvxTYPpt6l8z1GppazEh4xWVju121andseZ-lSvsICDYXQyv57yJUFrp9gjywbJ8zHvOhg6eKw-dQ</t>
+        </is>
+      </c>
+      <c r="L715" t="inlineStr">
+        <is>
+          <t>Arkseiro is back#rumi</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>Pouzitoz</t>
+        </is>
+      </c>
+      <c r="H716" t="inlineStr">
+        <is>
+          <t>fei_last_dance</t>
+        </is>
+      </c>
+      <c r="I716" t="inlineStr">
+        <is>
+          <t>DoylJ0gxSeT4yyyzit84eBFgjU6sJpTulGyF2J64I402SvQf2gk_UjxlOYpipB_DDpWsRBuC_Ko5Yw</t>
+        </is>
+      </c>
+      <c r="L716" t="inlineStr">
+        <is>
+          <t>Pouzitoz#blob</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>kauewrx</t>
+        </is>
+      </c>
+      <c r="H717" t="inlineStr">
+        <is>
+          <t>fei_last_dance</t>
+        </is>
+      </c>
+      <c r="I717" t="inlineStr">
+        <is>
+          <t>n8JyqP9LI6b4LuB54kZa6Ba6P04P1DvUeiwwZ8iyrw3qWXnvqgtRnPzbLL0l3hyuq4mzHJ6ur3l7cg</t>
+        </is>
+      </c>
+      <c r="L717" t="inlineStr">
+        <is>
+          <t>Subaru Wrx 2003#EJ207</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>cesinhas</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>ufu_saints_onyx</t>
+        </is>
+      </c>
+      <c r="G718" t="inlineStr">
+        <is>
+          <t>ufu_saints_onyx</t>
+        </is>
+      </c>
+      <c r="I718" t="inlineStr">
+        <is>
+          <t>W2PKpN-JzNrW48uv-plldpeSgcLtKJsI30vUCExwyoKKlx9hvLZro-r_1Wi0y1Wl5DkCdGxzSzHIZg</t>
+        </is>
+      </c>
+      <c r="L718" t="inlineStr">
+        <is>
+          <t>Chico Amaro#mari</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>Karbonick</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="G719" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="I719" t="inlineStr">
+        <is>
+          <t>ouJiodE8Muw_axHMln0MybsuW1tGdpflgnx-S-RyPk8b2fA8Kaa0IiyX0XsD7HQzsUfG5e4UMKbyOA</t>
+        </is>
+      </c>
+      <c r="L719" t="inlineStr">
+        <is>
+          <t>Karbonick#CO2</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>phmvasc</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="G720" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="I720" t="inlineStr">
+        <is>
+          <t>s-ZShvnVUEJjPukjN3RmZQk0POmIRdd-VPeuVVPwtoeeBfRdhzRZyVMeLlzfZKKXG8X9tZzJBm-XhA</t>
+        </is>
+      </c>
+      <c r="L720" t="inlineStr">
+        <is>
+          <t>phmvasc#KING</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Temmonn</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="G721" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="I721" t="inlineStr">
+        <is>
+          <t>CLygvtCeDHAA4oUSTTfVSr8_m1t316Y6JoOSA_NdX7PzXLpQzn-_OaTOg5yWnQeDIfaTe-G3L1vuGQ</t>
+        </is>
+      </c>
+      <c r="L721" t="inlineStr">
+        <is>
+          <t>AZR Temmonn#New</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Jacare</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="G722" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="I722" t="inlineStr">
+        <is>
+          <t>1BuisPlTAWPENS9iDbEzwo9xiArywALoHsc27jLmfUsDKoOuYX7pk8yQF4fAhsbfYfuaTwfslX82nw</t>
+        </is>
+      </c>
+      <c r="L722" t="inlineStr">
+        <is>
+          <t>Jacare#4638</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>GregorySouza</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="G723" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="I723" t="inlineStr">
+        <is>
+          <t>vtHoo8ZXrbs-Y_e_YIK8HDnfvyekn_5wEQFvZFbiy6Sd7iTaMQYgAx5kh7alOCIO_tunhoN9Dvk2zg</t>
+        </is>
+      </c>
+      <c r="L723" t="inlineStr">
+        <is>
+          <t>AlguemAi#AZR</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Cantarelli</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="G724" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="I724" t="inlineStr">
+        <is>
+          <t>LFV9Xqgum-P6oFl1ZL6wIAeAJkzoTkVV987aqo1Rmy6KAjFplCiLvr_dfdeeNz-CefKecLOqqHhGVw</t>
+        </is>
+      </c>
+      <c r="L724" t="inlineStr">
+        <is>
+          <t>Cantarelli#1722</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>MIRILO</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="G725" t="inlineStr">
+        <is>
+          <t>azure_bears_spotline</t>
+        </is>
+      </c>
+      <c r="I725" t="inlineStr">
+        <is>
+          <t>yR252lGhTu-ERmZOhn5yLNY9PI0w10zSVboTSu07BHve39ZRzlRkE9Bva7Qx6TWpDCPdzi9VVFcj4Q</t>
+        </is>
+      </c>
+      <c r="L725" t="inlineStr">
+        <is>
+          <t>MIRILO#NAJA</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>migzzz69</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>ufpr_bbn</t>
+        </is>
+      </c>
+      <c r="G726" t="inlineStr">
+        <is>
+          <t>ufpr_bbn</t>
+        </is>
+      </c>
+      <c r="I726" t="inlineStr">
+        <is>
+          <t>KodyjvJAbUcZ8bJGFJy2v4awUwC0cyUBy7v-ZlwPbp-WJhNryAXT72wej9spAqsGH1df9vqNrrLaXQ</t>
+        </is>
+      </c>
+      <c r="L726" t="inlineStr">
+        <is>
+          <t>little pank#jojix</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>f1lipinho</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>incinera_esports</t>
+        </is>
+      </c>
+      <c r="G727" t="inlineStr">
+        <is>
+          <t>incinera_esports</t>
+        </is>
+      </c>
+      <c r="I727" t="inlineStr">
+        <is>
+          <t>jlykeRy8jXd3LZpQRch0WBJOebEdm_1saYONr5vuMt3q5rsC0qVeH0il5sGnL9qwNHfPuS0H7E5bFw</t>
+        </is>
+      </c>
+      <c r="L727" t="inlineStr">
+        <is>
+          <t>hate javascript#sleep</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>ari$e</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>incinera_esports</t>
+        </is>
+      </c>
+      <c r="G728" t="inlineStr">
+        <is>
+          <t>incinera_esports</t>
+        </is>
+      </c>
+      <c r="I728" t="inlineStr">
+        <is>
+          <t>Eu33nG7HnbAR22y8NnzPfW1qWsxDuLj-Rg0Q20oAZuvqgT-VVntXLRx7qOVVB7X7iWVxb7K2z6Ag7w</t>
+        </is>
+      </c>
+      <c r="L728" t="inlineStr">
+        <is>
+          <t>black jesus#lila</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>typeshii</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="G729" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="I729" t="inlineStr">
+        <is>
+          <t>_Tdnb8qXlm3eyDKJcXuvudrRAXIGla18iAUHPVmYWmV67NVHyUy4y-AcVZpbjry3J_qiY8yd6E1ppQ</t>
+        </is>
+      </c>
+      <c r="L729" t="inlineStr">
+        <is>
+          <t>type shi#0000</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>chikao</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="G730" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="I730" t="inlineStr">
+        <is>
+          <t>Yl5gBlCdk1hKcPvtNUzQ_-06ed3FiUhVqLTo43iGOMmG2voHZBj3lqwxwZpmvBsCcJMgT2zNn22rHQ</t>
+        </is>
+      </c>
+      <c r="L730" t="inlineStr">
+        <is>
+          <t>chikao#0330</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>giga</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="G731" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="I731" t="inlineStr">
+        <is>
+          <t>oQGjzrREuX8HTrqWLN_LNNrIsIniUGIQFHsr09mRijvY5J7kyccgicUd-wWgF2FZ6eeJGfA16bgisA</t>
+        </is>
+      </c>
+      <c r="L731" t="inlineStr">
+        <is>
+          <t>giga#9790</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>Solium</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="G732" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="I732" t="inlineStr">
+        <is>
+          <t>Fv5xgLCpIEM8nwQZIKJ18NyDKAbclR-_5fHKNdC537OIrKdIWcM7BuFuSLhZIxk8rHMQPe_wVH_b8A</t>
+        </is>
+      </c>
+      <c r="L732" t="inlineStr">
+        <is>
+          <t>Solium#sdzy</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>ssob</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="G733" t="inlineStr">
+        <is>
+          <t>azure_bears_polaris</t>
+        </is>
+      </c>
+      <c r="I733" t="inlineStr">
+        <is>
+          <t>Y64aI23z1EbKJgo42AvENPuvlybggQ16eE6Owt9M_5wrjjAlOw6hx9kILX5F-O5zYZV90q8VCb8lFQ</t>
+        </is>
+      </c>
+      <c r="L733" t="inlineStr">
+        <is>
+          <t>ssob#永遠28</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>JuHornet</t>
+        </is>
+      </c>
+      <c r="H734" t="inlineStr">
+        <is>
+          <t>macklogic_wine</t>
+        </is>
+      </c>
+      <c r="I734" t="inlineStr">
+        <is>
+          <t>rRyXlRlM15UiKQXjqkoBh3DSxwia6Yk8eDcb6qN7yaFqkfveyyksYzkC_tZvDBJsjn-gIbxQK_3p-w</t>
+        </is>
+      </c>
+      <c r="L734" t="inlineStr">
+        <is>
+          <t>237 JuHornet#YKGG</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>DrogaeoTL</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="G735" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="I735" t="inlineStr">
+        <is>
+          <t>XNXAEXFANPa_Iu2bQ2yEOKwZsLZoVHhUGMK7rwAJR76fWAWzXDrI33exxol5YtEGsQCRj66rmAlP9g</t>
+        </is>
+      </c>
+      <c r="L735" t="inlineStr">
+        <is>
+          <t>DrogaéoTL#999</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>Daske</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="G736" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="I736" t="inlineStr">
+        <is>
+          <t>YxhqrMTfJPwiamZD6LzTGMMDngG9hg7P98PB6lsPgWQVf_XpDAucgXMkZvPFQXNOi9cKvru5Z_1XqA</t>
+        </is>
+      </c>
+      <c r="L736" t="inlineStr">
+        <is>
+          <t>Daske#MDM</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>gabribs</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="G737" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="I737" t="inlineStr">
+        <is>
+          <t>h_o3l9TA7jnt1Ib7lmGjYhWKoFsWnGiwYW9eEKWlGlhX96JrbdSisAVtJgjfhFDlGkyONs9F7WOC8A</t>
+        </is>
+      </c>
+      <c r="L737" t="inlineStr">
+        <is>
+          <t>you belong to me#0906</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>BlackCat</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="G738" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="I738" t="inlineStr">
+        <is>
+          <t>dJVDh2HQ6cYZfg01TYvpzyPN1FJYt2I61e_oK1LLJctEDG0xvCCYmXkPet3JS6rcIiRiXKWSQiNo5w</t>
+        </is>
+      </c>
+      <c r="L738" t="inlineStr">
+        <is>
+          <t>BlackCat黒猫#3035</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>caiotif</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="G739" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="I739" t="inlineStr">
+        <is>
+          <t>Og1LoqH6b98DaYiu8Yb29wRQQOgAE7l1iS86k69tEH-pEPkIIIAJq3XA-ovATqLx394IczEvu-b6yw</t>
+        </is>
+      </c>
+      <c r="L739" t="inlineStr">
+        <is>
+          <t>unknown#scars</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>art3mis</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="G740" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="I740" t="inlineStr">
+        <is>
+          <t>_eNAwYFIjong_F4UDZ_NXqMfc8KsXo6RjgYkaHIyP6xOChBcpT1yWBuCumOemACKAdfPxQnRafgWWQ</t>
+        </is>
+      </c>
+      <c r="L740" t="inlineStr">
+        <is>
+          <t>artemis#1984</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>zelax</t>
+        </is>
+      </c>
+      <c r="H741" t="inlineStr">
+        <is>
+          <t>atletica_sustenta</t>
+        </is>
+      </c>
+      <c r="I741" t="inlineStr">
+        <is>
+          <t>LQ-wX2xPRwPu4U43F0dagGS6qm_4Try_Rl30vOtTBvKSgoiTOPku3oRIHkDXFSlBuk8N1Cjae6k6_w</t>
+        </is>
+      </c>
+      <c r="L741" t="inlineStr">
+        <is>
+          <t>britadeira#Klebe</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>iguin</t>
+        </is>
+      </c>
+      <c r="H742" t="inlineStr">
+        <is>
+          <t>atletica_sustenta</t>
+        </is>
+      </c>
+      <c r="I742" t="inlineStr">
+        <is>
+          <t>Hcg1ZKKgRKIm_v4QJWNalOa7jkFxyF34-o3ivg0NPFEEkZlBwzxpk4EPfkE52PvKmUEX1gxwVZyKJg</t>
+        </is>
+      </c>
+      <c r="L742" t="inlineStr">
+        <is>
+          <t>iguin dos prédio#kaká</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>NICCKK</t>
+        </is>
+      </c>
+      <c r="H743" t="inlineStr">
+        <is>
+          <t>atletica_sustenta</t>
+        </is>
+      </c>
+      <c r="I743" t="inlineStr">
+        <is>
+          <t>FjrMogJRHo7QMWI-59no0K0eWaVydtxc0f3USpeD2dow3U8Z5JLK7QL3KKDQ8Ijtiphq5jj2iN6fZw</t>
+        </is>
+      </c>
+      <c r="L743" t="inlineStr">
+        <is>
+          <t>NICCKK#uwu</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>Milanga</t>
+        </is>
+      </c>
+      <c r="H744" t="inlineStr">
+        <is>
+          <t>fei_last_dance</t>
+        </is>
+      </c>
+      <c r="I744" t="inlineStr">
+        <is>
+          <t>oktjrpu0nX6ydevJIMGtfyPzyyLSEbQe9M9EvKScL6a6oIYjO-AOdTKNvIKJ4Y1Yt7V7XBrL7uHDqw</t>
+        </is>
+      </c>
+      <c r="L744" t="inlineStr">
+        <is>
+          <t>TRP Milanga#Gordo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
astra cup e e-tusca no site, com cadastro e icones
- Astra Cup Inclusivo (AcadArena, presencial, 10/10): pontos corridos MD1
  com 4 equipes. Rainbow 3-0, Canaries 2-1, USP 1-2, INATEL 0-3.
- E-Tusca 2026 (AcadArena, 27/09 e 04/10): suico de 2 rodadas e playoffs
  MD3, desenhado como chave. Final PUCC Cardinals 2x1 AXIS, como nos
  arquivos (a plataforma inverteu o 3o mapa; o dono confirmou a PUCC).
- Decisoes do dono: LAP PUCCAMPINAS = PUCC Cardinals, Canaries SANJA = PUCC
  Canaries, os dois no tier B, pontos como o Pre-JUBS SP (20/15/10/5).
- Cadastro: 6 contas novas que jogaram, PUUID da Bielorrusia, 9 nicks novos
  (cada um conferido pelo PUUID), Nacaguma com current_team na Cardinals e
  completes para Violetx e lule.
- Icones AstraCup.png e tusca.png otimizados; capa e trofeu genericos.

Ranking: mudam os cortes a partir de 29/09. PUCC Cardinals 15o -> 9o e
MackLogic Rainbow entra em 24o.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/dados_excel/players.xlsx
+++ b/dados_excel/players.xlsx
@@ -466,7 +466,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q744"/>
+  <dimension ref="A1:Q750"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="24" defaultRowHeight="14.4"/>
   <cols>
     <col width="15.6640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1042,6 +1042,11 @@
           <t>thaly#gus</t>
         </is>
       </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>thaly#2302</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1140,9 +1145,19 @@
           <t>usp_stars_gc</t>
         </is>
       </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>tAWTzpnPhLlsbGEYyNjIYcOm63rdaGGWGIMWrAvTCqSyR-ZI0gNvHsdH5fy37ddMcDIsPN0sZDnp6g</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>Bielorrússia#gaay</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Bielorrússia#fflch</t>
         </is>
       </c>
     </row>
@@ -4085,6 +4100,11 @@
           <t>anakin#gbxz</t>
         </is>
       </c>
+      <c r="M122" t="inlineStr">
+        <is>
+          <t>gbxz1#goldb</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -7957,6 +7977,11 @@
           <t>PUCC ttt#ttt</t>
         </is>
       </c>
+      <c r="N258" t="inlineStr">
+        <is>
+          <t>maldi sinistrão#anna</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
@@ -8139,6 +8164,11 @@
           <t>é o maldito#crstl</t>
         </is>
       </c>
+      <c r="O264" t="inlineStr">
+        <is>
+          <t>Ti da PUCC#mafe</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -9899,7 +9929,7 @@
       </c>
       <c r="H323" t="inlineStr">
         <is>
-          <t>macklogic_wine</t>
+          <t>macklogic_wine;macklogic_rainbow</t>
         </is>
       </c>
       <c r="I323" t="inlineStr">
@@ -10084,6 +10114,11 @@
           <t>Sea#yuumi</t>
         </is>
       </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>Sea#dora</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -14914,6 +14949,11 @@
           <t>Zorua fanboy#lizi</t>
         </is>
       </c>
+      <c r="N489" t="inlineStr">
+        <is>
+          <t>Abyss Star#death</t>
+        </is>
+      </c>
     </row>
     <row r="490">
       <c r="A490" t="inlineStr">
@@ -15135,6 +15175,11 @@
           <t>caap_auroras</t>
         </is>
       </c>
+      <c r="H497" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
       <c r="I497" t="inlineStr">
         <is>
           <t>zcRFQ5ldWqETHkJqN0L6meOnVAOE8d1KKueLCWOILAT5olCXgImIJdZmPlFKQTbFpXEYsW6LotWmdw</t>
@@ -16543,6 +16588,11 @@
           <t>Zé Drops#sara</t>
         </is>
       </c>
+      <c r="N541" t="inlineStr">
+        <is>
+          <t>Zé Kushala#sara</t>
+        </is>
+      </c>
     </row>
     <row r="542">
       <c r="A542" t="inlineStr">
@@ -16585,6 +16635,11 @@
           <t>demonicks#nath</t>
         </is>
       </c>
+      <c r="N542" t="inlineStr">
+        <is>
+          <t>nicks#peace</t>
+        </is>
+      </c>
     </row>
     <row r="543">
       <c r="A543" t="inlineStr">
@@ -16654,6 +16709,11 @@
           <t>vladi#juubs</t>
         </is>
       </c>
+      <c r="M544" t="inlineStr">
+        <is>
+          <t>vladi iwnl#juubs</t>
+        </is>
+      </c>
     </row>
     <row r="545">
       <c r="A545" t="inlineStr">
@@ -18372,6 +18432,11 @@
           <t>pucc_cardinals</t>
         </is>
       </c>
+      <c r="G603" t="inlineStr">
+        <is>
+          <t>pucc_cardinals</t>
+        </is>
+      </c>
       <c r="I603" t="inlineStr">
         <is>
           <t>W6PWu2QLZLVd7m48FXH3vY2Y9i3slF_v9s9Yf2QD_SCLZu5zyI3sSQzf-k65O7XFadAKhSCHiOceLw</t>
@@ -22162,6 +22227,168 @@
       <c r="L744" t="inlineStr">
         <is>
           <t>TRP Milanga#Gordo</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>NoobViciada</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>usp_stars_gc</t>
+        </is>
+      </c>
+      <c r="G745" t="inlineStr">
+        <is>
+          <t>usp_stars_gc</t>
+        </is>
+      </c>
+      <c r="I745" t="inlineStr">
+        <is>
+          <t>fnecMmOa1KHgtS0YfrH6XCs6cPDELSGjTLFWv_h7NMrOHpoDGE28QnNc44TC8pLSAjT7_6OaybIIpA</t>
+        </is>
+      </c>
+      <c r="L745" t="inlineStr">
+        <is>
+          <t>NoobViciada#br1</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>aimeeaimee</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="G746" t="inlineStr">
+        <is>
+          <t>pucc_canaries</t>
+        </is>
+      </c>
+      <c r="I746" t="inlineStr">
+        <is>
+          <t>tys0cdsFtvvTPnm_UPSZb4ZmdHFb4FnGHAgUs6LXCkNLRLCcajy14jUq37M2dYuDKUv8cK1_Uc4P_A</t>
+        </is>
+      </c>
+      <c r="L746" t="inlineStr">
+        <is>
+          <t>starfire#1606</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>Mdz</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>unicamp_tritons_black</t>
+        </is>
+      </c>
+      <c r="G747" t="inlineStr">
+        <is>
+          <t>unicamp_tritons_black</t>
+        </is>
+      </c>
+      <c r="I747" t="inlineStr">
+        <is>
+          <t>96fH2sGFsgNOsId_tcw8BO2XZ1khJ-bdW37MOLBc0mDJQY9fMeCbEVeLUa9npadHKIfkL46g4kTYQw</t>
+        </is>
+      </c>
+      <c r="L747" t="inlineStr">
+        <is>
+          <t>Mdz#6661</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>BigaBigato</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="G748" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="I748" t="inlineStr">
+        <is>
+          <t>kLHSLMMNnu-aWPXWJfhlPzag9fH_tGyO8A5X-Q-awzf7E7g2CXSgaDqWVYxBbjJLUUclBXpu6GJMHg</t>
+        </is>
+      </c>
+      <c r="L748" t="inlineStr">
+        <is>
+          <t>Brida Nunes#prvcy</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>Thigas</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="G749" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="I749" t="inlineStr">
+        <is>
+          <t>dz6ZvyB82m3suKGgqjS5QkdC9HdNDMKeAdVEHQdAv-gWSTYl0IWtBlP6nZcFV1HVK3IMD-p3PvNqhg</t>
+        </is>
+      </c>
+      <c r="L749" t="inlineStr">
+        <is>
+          <t>Thigas#000</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>nobukuni</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="G750" t="inlineStr">
+        <is>
+          <t>ufscar_fire</t>
+        </is>
+      </c>
+      <c r="I750" t="inlineStr">
+        <is>
+          <t>n28tm2-7yrTZ0wFlj3dS3rPK_pvyOe6kus_zq6YEPx1TyPw5wec9TgD5sQYLmknt4Qyf9uYUsMvuRA</t>
+        </is>
+      </c>
+      <c r="L750" t="inlineStr">
+        <is>
+          <t>CarrinhoDePirok#br1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Preserve current local site as editorial design baseline
</commit_message>
<xml_diff>
--- a/dados_excel/players.xlsx
+++ b/dados_excel/players.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -941,11 +941,6 @@
           <t>wolf_gaming</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>wolf_gaming</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>u9ICdhbvgpXi42XhszYP0F1LscHkpiee1a2DApmiP0OzsI98RdWD8mcygA1-IlPQIxVb8deraS_KXw</t>
@@ -1140,11 +1135,6 @@
           <t>usp_stars_gc</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>usp_stars_gc</t>
-        </is>
-      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>tAWTzpnPhLlsbGEYyNjIYcOm63rdaGGWGIMWrAvTCqSyR-ZI0gNvHsdH5fy37ddMcDIsPN0sZDnp6g</t>
@@ -1172,11 +1162,6 @@
           <t>usp_stars_gc</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>usp_stars_gc</t>
-        </is>
-      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>_WZpUmN7nBBFJ_MbGLditmDFthPf61fdPnYCei0g800r9lpc2My0rN31Dzoy4A_sbXIYGJ93wzSFMg</t>
@@ -1253,11 +1238,6 @@
           <t>usp_stars</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>usp_stars</t>
-        </is>
-      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>mEl8mUKuDxynBb38jXsHTBnE6F-z2OUzk8PKpKljnHcT1PRnkWKFM44I3ZxXLHUItzz6DOhi9ksSyA</t>
@@ -2309,11 +2289,6 @@
           <t>unirio_krakens</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>unirio_krakens</t>
-        </is>
-      </c>
       <c r="I64" t="inlineStr">
         <is>
           <t>Utp2yVXMV4mmUCo09_RcsF64VrOXnIqBtyA_-kE_UBXqKvib8yyFYMX8nAze_UKK4Z56ngWTSMe1NA</t>
@@ -3288,11 +3263,6 @@
           <t>unicamp_tritons_black</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>unicamp_tritons_black</t>
-        </is>
-      </c>
       <c r="I96" t="inlineStr">
         <is>
           <t>88G6xgaAAef5qemLkAbm_UEo1nWCPnK1V7WQBy49e1BS4cCCAVOi16Ml33pCXqu6FrPnfVZu6c--QA</t>
@@ -3903,11 +3873,6 @@
           <t>ufu_saints</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>ufu_saints</t>
-        </is>
-      </c>
       <c r="I116" t="inlineStr">
         <is>
           <t>PUcyfXweL2QkiapM6bxnyPCweB-ITtYFQHvdfkcSOPl1R0zdfUEgN7W0zs4M13zvj15XRUFd7W_GpQ</t>
@@ -3930,11 +3895,6 @@
           <t>ufu_saints</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>ufu_saints</t>
-        </is>
-      </c>
       <c r="I117" t="inlineStr">
         <is>
           <t>jfvKJJQmJ3vOg5rEUYN9Z67ibW2jnXGoQVITcE1IwK35-nsHLENNTnAN1npg0dzHUYERMrvzFbSM4A</t>
@@ -4058,11 +4018,6 @@
           <t>ufscar_fire</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>ufscar_fire</t>
-        </is>
-      </c>
       <c r="I121" t="inlineStr">
         <is>
           <t>bKsWXR9kAaZTMFmUA8Da_oBmzfFpE8JeS6QKFTUTmUprc8RSpLIw2FNBYRZNVpomvRshJzo1GI5S1g</t>
@@ -4626,11 +4581,6 @@
           <t>ufrj_minerva</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>ufrj_minerva</t>
-        </is>
-      </c>
       <c r="I140" t="inlineStr">
         <is>
           <t>im4BHDdELr1YKI4fX4mx9xS4hI-7SLWjsv8w16mAnyhyyylhbNh6jS_VtNuGIZjI-mZfZUddHWDLCA</t>
@@ -4948,11 +4898,6 @@
           <t>ufpr_bbn</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>ufpr_bbn</t>
-        </is>
-      </c>
       <c r="I151" t="inlineStr">
         <is>
           <t>bKYcnZJ-ToLmXHs45QuEJV7tdqCUIoMEU5-vFzBsAogC9VGqFN9puYwigg6JKcVd5caFm4145uN1lg</t>
@@ -4975,11 +4920,6 @@
           <t>ufpr_bbn</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>ufpr_bbn</t>
-        </is>
-      </c>
       <c r="I152" t="inlineStr">
         <is>
           <t>g-IvHtnI6kdiFnRFVnSVmtzKk8uZF4tulJpTcoqMe7tFgw5GXPJZ7xD7KxlfvqrJac5YHrRB7jYaTQ</t>
@@ -5179,11 +5119,6 @@
           <t>ufmt_turuna</t>
         </is>
       </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>ufmt_turuna</t>
-        </is>
-      </c>
       <c r="I159" t="inlineStr">
         <is>
           <t>WbmDscUxGUIMc2mq9e0W3SKTMxsMQL9xJ_P3jrFy4B5BATZ_9OaaUwDwznw2bFoBkZVnv6leOlzbpA</t>
@@ -6984,11 +6919,6 @@
           <t>totale_umc</t>
         </is>
       </c>
-      <c r="G224" t="inlineStr">
-        <is>
-          <t>totale_umc</t>
-        </is>
-      </c>
       <c r="I224" t="inlineStr">
         <is>
           <t>DEHyORp293uMthwlUKVrqEY7oQk3GK6YkM57y0eenYaqqZH4ZwBsRdZULpZth5GDPPB1s3kX6meaDQ</t>
@@ -7694,11 +7624,6 @@
           <t>pucgo_sistematica</t>
         </is>
       </c>
-      <c r="G249" t="inlineStr">
-        <is>
-          <t>pucgo_sistematica</t>
-        </is>
-      </c>
       <c r="I249" t="inlineStr">
         <is>
           <t>Plj4rlGsRBSkIKnfisJi-MV2sepg3SpaxRB98OoGga07acGP2eVLbgLqLIYxQjYeKc82FRlMFqkcrg</t>
@@ -7780,11 +7705,6 @@
           <t>pucgo_sistematica</t>
         </is>
       </c>
-      <c r="G252" t="inlineStr">
-        <is>
-          <t>pucgo_sistematica</t>
-        </is>
-      </c>
       <c r="I252" t="inlineStr">
         <is>
           <t>P8aY38Slk3RKg60vPOCKSsWTDmFKMsN6eTJjQLnUxvvwOgW33hejt3vmLnCKCncWxyoNmS7TO9i0gQ</t>
@@ -7834,11 +7754,6 @@
           <t>pucgo_sistematica</t>
         </is>
       </c>
-      <c r="G254" t="inlineStr">
-        <is>
-          <t>pucgo_sistematica</t>
-        </is>
-      </c>
       <c r="I254" t="inlineStr">
         <is>
           <t>dcX1EoCibLxmHNZRAyBwY-r81ItkAZe5NX2TtQXwbgY-YUdXSKSplOm7hL9pS-ftYB_ggFGkKY1Vhg</t>
@@ -7920,11 +7835,6 @@
           <t>pucc_cardinals</t>
         </is>
       </c>
-      <c r="G257" t="inlineStr">
-        <is>
-          <t>pucc_cardinals</t>
-        </is>
-      </c>
       <c r="I257" t="inlineStr">
         <is>
           <t>301qhx0vRdUVcofBGyq_VoAhuOwFm2GLKQ93asIyj37qjY-dG2lzyjNQHKIalkgRT4G9l7htJmVQkQ</t>
@@ -8053,11 +7963,6 @@
           <t>pucc_cardinals</t>
         </is>
       </c>
-      <c r="G261" t="inlineStr">
-        <is>
-          <t>pucc_cardinals</t>
-        </is>
-      </c>
       <c r="I261" t="inlineStr">
         <is>
           <t>ua9cSJ_WLHTDUhQhJYjkWcZ20qEiMBblpkY2SUuGfXrZij10AMpGNKivg1OCuCWXcJL5XN6ZNTcHcQ</t>
@@ -8080,11 +7985,6 @@
           <t>pucc_cardinals</t>
         </is>
       </c>
-      <c r="G262" t="inlineStr">
-        <is>
-          <t>pucc_cardinals</t>
-        </is>
-      </c>
       <c r="I262" t="inlineStr">
         <is>
           <t>QAn49vDOOkmlsACPBxsDlBH-p5bl93HPVr0DwAcwsPoqOEthQdSKL_2-ecm5IlT2uVxv52uuVrW4ew</t>
@@ -9437,11 +9337,6 @@
           <t>maua_blue</t>
         </is>
       </c>
-      <c r="G308" t="inlineStr">
-        <is>
-          <t>maua_blue</t>
-        </is>
-      </c>
       <c r="I308" t="inlineStr">
         <is>
           <t>HnS2m2EByAsSUFVsmd4FLWmlzRdtYLiURpHDpTYXYGZp6XS1YHKzXjPiBEe-biZAOcknSGbEcXyQ8w</t>
@@ -9464,11 +9359,6 @@
           <t>maua_blue</t>
         </is>
       </c>
-      <c r="G309" t="inlineStr">
-        <is>
-          <t>maua_blue</t>
-        </is>
-      </c>
       <c r="I309" t="inlineStr">
         <is>
           <t>5DtyRi2zT34YBGF66FSePkScbdKjEW9pPNB_aguFegUuHPK9kOvny5ZtfQfgzSYJgEEMjxDsiBMisA</t>
@@ -9518,11 +9408,6 @@
           <t>maua_blue</t>
         </is>
       </c>
-      <c r="G311" t="inlineStr">
-        <is>
-          <t>maua_blue</t>
-        </is>
-      </c>
       <c r="I311" t="inlineStr">
         <is>
           <t>gaSDlUryf--PXz557skg2GMkc2tLsessde_L76p-ArFgiId0mCbsPSnaDzS-mYuKT3MZiyBRNK_2Hg</t>
@@ -9577,11 +9462,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G313" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I313" t="inlineStr">
         <is>
           <t>2yslosTvB5-Q9mszSTYnUsHkt8dc2ryhnysRiaa_oUw7t3C45vaUQOWzro4OUYgztuiNKwu9zoaYtA</t>
@@ -9609,11 +9489,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G314" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I314" t="inlineStr">
         <is>
           <t>9edCRwvelp9Ko7rrbtTbk86da6un1VgQVZ7HFf0x3G8hmQbpGxGkY1D9QBQOYECuAHROjMACZxeW-g</t>
@@ -9636,11 +9511,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G315" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I315" t="inlineStr">
         <is>
           <t>DgRoFzXydtAKcOh2ntoyp6iqGyAOgMG3CWFcXnYTmmoGnijHaKCFS_u8tT47bILJOS8V_0mqSyVw2A</t>
@@ -9742,11 +9612,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G318" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I318" t="inlineStr">
         <is>
           <t>-SEFIRD9iWcerWPwSbl2xqpiq2BWZnWrBz8ZbT0Wl4-QpQ_LTtAxbBW_Y3qAdL9dr-EJPrQCQg5dtg</t>
@@ -9769,11 +9634,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G319" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I319" t="inlineStr">
         <is>
           <t>zUF3dytt7KB_gS05Zkpnmjb138wJb3onG45XJIDiMnS4m3NbY8dpaXSSfPCJGRvx0Gq4ZAOcliMayA</t>
@@ -9796,11 +9656,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G320" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="H320" t="inlineStr">
         <is>
           <t>macklogic_red; macklogic_wine</t>
@@ -9986,11 +9841,6 @@
           <t>macklogic_red</t>
         </is>
       </c>
-      <c r="G325" t="inlineStr">
-        <is>
-          <t>macklogic_red</t>
-        </is>
-      </c>
       <c r="I325" t="inlineStr">
         <is>
           <t>UMqsz421_7TZxaMOWSfkHTe8pC3sApewo-dX9I-Em4VbL0PwyTh6QNaYOT2chpOseS1UmfxTl9zkNQ</t>
@@ -10131,11 +9981,6 @@
           <t>macklogic_rainbow</t>
         </is>
       </c>
-      <c r="G330" t="inlineStr">
-        <is>
-          <t>macklogic_rainbow</t>
-        </is>
-      </c>
       <c r="I330" t="inlineStr">
         <is>
           <t>w8dgJVfD_Y64jJfKQRN8eKJNmxOeCnJEZnuGgJs5rlG3a_zdNycRrHlLyMw4ryNLeNoRai8a5jcA5A</t>
@@ -11057,11 +10902,6 @@
           <t>inatel_gray</t>
         </is>
       </c>
-      <c r="G363" t="inlineStr">
-        <is>
-          <t>inatel_gray</t>
-        </is>
-      </c>
       <c r="I363" t="inlineStr">
         <is>
           <t>PD2xOUFZLkq-i7-2FyDihzZEZNZtqNraY5XhJ0CqsB6WhXK9s-VtLuXy7dCepywKEjXgyyVPYp2Mvg</t>
@@ -11084,11 +10924,6 @@
           <t>inatel_gray</t>
         </is>
       </c>
-      <c r="G364" t="inlineStr">
-        <is>
-          <t>inatel_gray</t>
-        </is>
-      </c>
       <c r="I364" t="inlineStr">
         <is>
           <t>azLzX0-fc5yL96eqiV6QbzK6TmuOBf31YuoUScb0ELyWswIQDLOLoY5MbijUYfnGqUmJ-xqH_Odg-A</t>
@@ -12551,11 +12386,6 @@
           <t>green_owls_noctua</t>
         </is>
       </c>
-      <c r="G415" t="inlineStr">
-        <is>
-          <t>green_owls_noctua</t>
-        </is>
-      </c>
       <c r="I415" t="inlineStr">
         <is>
           <t>21R3F3xWR-kcyY9bP3cg684JI--MG0f3wv3loFoQPtR19ojbhniQ07Tr3yUusAi-ZoDgqs-rCMlR4Q</t>
@@ -12880,11 +12710,6 @@
           <t>gambiarra_ufg</t>
         </is>
       </c>
-      <c r="G427" t="inlineStr">
-        <is>
-          <t>gambiarra_ufg</t>
-        </is>
-      </c>
       <c r="L427" t="inlineStr">
         <is>
           <t>Thorfinn メ#naves</t>
@@ -12983,11 +12808,6 @@
           <t>furia_utfpr</t>
         </is>
       </c>
-      <c r="G431" t="inlineStr">
-        <is>
-          <t>furia_utfpr</t>
-        </is>
-      </c>
       <c r="I431" t="inlineStr">
         <is>
           <t>gfM9fyh51WHYAr4dX7Rnds0UKwEY3WfPFsncjdfcxYTE9s2NbsmzxurTn76dKcuXhwygOj3WR_EKjA</t>
@@ -14012,11 +13832,6 @@
           <t>ceub_octopus_vulgaris</t>
         </is>
       </c>
-      <c r="G463" t="inlineStr">
-        <is>
-          <t>ceub_octopus_vulgaris</t>
-        </is>
-      </c>
       <c r="H463" t="inlineStr">
         <is>
           <t>atletica_sustenta</t>
@@ -14801,11 +14616,6 @@
           <t>caap_malditos</t>
         </is>
       </c>
-      <c r="G485" t="inlineStr">
-        <is>
-          <t>caap_malditos</t>
-        </is>
-      </c>
       <c r="I485" t="inlineStr">
         <is>
           <t>E3ivYGaicB2XlnMhnolVgM0wf7s-1z7f3Xq8YCQtFgMsBw-I8ZFrfKmDgEeh7kD_k7P_AdfFuR20kg</t>
@@ -14966,11 +14776,6 @@
           <t>caap_hellhounds</t>
         </is>
       </c>
-      <c r="G490" t="inlineStr">
-        <is>
-          <t>caap_hellhounds</t>
-        </is>
-      </c>
       <c r="I490" t="inlineStr">
         <is>
           <t>_IMaT7l5138--TeO3kpZ_7ejIV_w32dNUnEmeJKzvNzh5KmslemzFZTQbydqibFW5ZHhifd-lcz54A</t>
@@ -15089,11 +14894,6 @@
           <t>caap_hellhounds</t>
         </is>
       </c>
-      <c r="G494" t="inlineStr">
-        <is>
-          <t>caap_hellhounds</t>
-        </is>
-      </c>
       <c r="I494" t="inlineStr">
         <is>
           <t>s_smSLBfGMdCnHDxwP0T0RFjRniaOr__qw72D73JzF7p4GXYPQx2qwbD2ILlrDsXPipLSplt3taL5Q</t>
@@ -15116,11 +14916,6 @@
           <t>caap_hellhounds</t>
         </is>
       </c>
-      <c r="G495" t="inlineStr">
-        <is>
-          <t>caap_hellhounds</t>
-        </is>
-      </c>
       <c r="I495" t="inlineStr">
         <is>
           <t>-k4zx9RhoxLQNGaEEVA4rw9o9_0HC-orLXCLIUtxJ0y8_-thVKLDNhfT1Ea-AGnXsOa0Nd0shSioYg</t>
@@ -15143,11 +14938,6 @@
           <t>caap_auroras</t>
         </is>
       </c>
-      <c r="G496" t="inlineStr">
-        <is>
-          <t>caap_auroras</t>
-        </is>
-      </c>
       <c r="I496" t="inlineStr">
         <is>
           <t>9gI-LexrKcJkxI1-xWQqbRSN8SwVvz3lwY3h0xBip886cf5g8L0sVQ9NogF70PfYCgb2VUy9HMJXsg</t>
@@ -15271,11 +15061,6 @@
           <t>caap_auroras</t>
         </is>
       </c>
-      <c r="G500" t="inlineStr">
-        <is>
-          <t>caap_auroras</t>
-        </is>
-      </c>
       <c r="I500" t="inlineStr">
         <is>
           <t>6jBTCJWXhj2d2kq6cTNjE3ykg55HXWJn0BHp59Yb_ukHkkflQn8JYca_mmFdESMmZI3jW94mEOdU8Q</t>
@@ -15753,11 +15538,6 @@
           <t>azure_bears_silver</t>
         </is>
       </c>
-      <c r="G516" t="inlineStr">
-        <is>
-          <t>azure_bears_silver</t>
-        </is>
-      </c>
       <c r="I516" t="inlineStr">
         <is>
           <t>FrflKIANQmKRQQTQPKmX0f8ZGnmo9n5eF42hWEDFL36laJkn_XbZX-u7VcHHNuOvsqMSgiKUc4zi9w</t>
@@ -15962,11 +15742,6 @@
           <t>azure_bears_golden</t>
         </is>
       </c>
-      <c r="G523" t="inlineStr">
-        <is>
-          <t>azure_bears_golden</t>
-        </is>
-      </c>
       <c r="I523" t="inlineStr">
         <is>
           <t>X6dK2xFXw4_isMR03zbzKl6bGGWP9X1kAFqdhsD4MV5qEcjArJhxIEiOp3xZP9fDpEUyCjNWTe2ajw</t>
@@ -16221,11 +15996,6 @@
           <t>azure_bears_black</t>
         </is>
       </c>
-      <c r="G530" t="inlineStr">
-        <is>
-          <t>azure_bears_black</t>
-        </is>
-      </c>
       <c r="I530" t="inlineStr">
         <is>
           <t>LBnUfrUKZa1Ry2fK1bWp7Ok0EizDW86Jd0jyt3FJJl044o3eS_2ZFcEICcjImD_Ow26oiKVSgFFvRg</t>
@@ -16610,11 +16380,6 @@
           <t>axis_anteaters</t>
         </is>
       </c>
-      <c r="G542" t="inlineStr">
-        <is>
-          <t>axis_anteaters</t>
-        </is>
-      </c>
       <c r="H542" t="inlineStr">
         <is>
           <t>sixa_eaters</t>
@@ -17445,11 +17210,6 @@
           <t>a2e_uff</t>
         </is>
       </c>
-      <c r="G567" t="inlineStr">
-        <is>
-          <t>a2e_uff</t>
-        </is>
-      </c>
       <c r="I567" t="inlineStr">
         <is>
           <t>YxfNWtbF20Z1tRTaFBSFyL1tHiLxkIV836jBLC96PNLp2lcAK-ZVauekN83dxgTq83Wdt6mwE4xUnQ</t>
@@ -17948,7 +17708,7 @@
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t>jotave</t>
+          <t>JotaVe</t>
         </is>
       </c>
       <c r="B585" t="inlineStr">
@@ -17963,7 +17723,7 @@
       </c>
       <c r="G585" t="inlineStr">
         <is>
-          <t>ceub_octopus_vulgaris</t>
+          <t>ceub_octopus</t>
         </is>
       </c>
       <c r="I585" t="inlineStr">
@@ -18121,11 +17881,6 @@
           <t>ceub_octopus_vulgaris</t>
         </is>
       </c>
-      <c r="G590" t="inlineStr">
-        <is>
-          <t>ceub_octopus_vulgaris</t>
-        </is>
-      </c>
       <c r="H590" t="inlineStr">
         <is>
           <t>atletica_sustenta</t>
@@ -18621,11 +18376,6 @@
           <t>ufu_saints</t>
         </is>
       </c>
-      <c r="G610" t="inlineStr">
-        <is>
-          <t>ufu_saints</t>
-        </is>
-      </c>
       <c r="I610" t="inlineStr">
         <is>
           <t>kVLPGLd0abwlSX6VkHzmWiuJtUe20TCvMaGG4R9bT6SezSyfhLjdcYO3gwzFMQciHDqNwOzQcfYkFg</t>
@@ -19499,11 +19249,6 @@
           <t>ufrj_minerva</t>
         </is>
       </c>
-      <c r="G644" t="inlineStr">
-        <is>
-          <t>ufrj_minerva</t>
-        </is>
-      </c>
       <c r="I644" t="inlineStr">
         <is>
           <t>6VmRqgEcADA3-FPKNyHudktkAmRCQ24f4-7qULqSetlt4BwhJOMPordrLxy5QW_H7xCbO87n8YDM4w</t>
@@ -19585,11 +19330,6 @@
           <t>ufrj_minerva</t>
         </is>
       </c>
-      <c r="G647" t="inlineStr">
-        <is>
-          <t>ufrj_minerva</t>
-        </is>
-      </c>
       <c r="I647" t="inlineStr">
         <is>
           <t>APM9XNdFLPZ0XIsxhQtKwlURG6MwycOF4EA0OZgJy-DCHEHh4vZmPDsjOjw2mUkEsJ-73BZEbseMrQ</t>
@@ -19774,11 +19514,6 @@
           <t>a2e_uff_shadows</t>
         </is>
       </c>
-      <c r="G654" t="inlineStr">
-        <is>
-          <t>a2e_uff_shadows</t>
-        </is>
-      </c>
       <c r="I654" t="inlineStr">
         <is>
           <t>K2nP5lhGeWcXKEoVzO1O-lICjLS4f2l_7X5U2uamQbAIxx3Jgkj_95sVV_ip-8TjWGrzQ1Yo4E049w</t>
@@ -19806,11 +19541,6 @@
           <t>a2e_uff</t>
         </is>
       </c>
-      <c r="G655" t="inlineStr">
-        <is>
-          <t>a2e_uff</t>
-        </is>
-      </c>
       <c r="I655" t="inlineStr">
         <is>
           <t>RRuFlSaUvwSAbsU0VZWUccWHztIDpZw_Q0uTHOpnzEfsCQUfxdzlNn3j5BEPEcQHEgwmSnmSfIzK1w</t>
@@ -20668,11 +20398,6 @@
           <t>brutal_esports</t>
         </is>
       </c>
-      <c r="G686" t="inlineStr">
-        <is>
-          <t>brutal_esports</t>
-        </is>
-      </c>
       <c r="I686" t="inlineStr">
         <is>
           <t>7Kip5H0Ns-j3RgPJqPL2CnGrSlwFygVFu8vG8IdWfuOVimmXaM-_kRhNAeipehmkzovgQGE5L80Ksw</t>
@@ -20695,11 +20420,6 @@
           <t>liga_vulkanica</t>
         </is>
       </c>
-      <c r="G687" t="inlineStr">
-        <is>
-          <t>liga_vulkanica</t>
-        </is>
-      </c>
       <c r="I687" t="inlineStr">
         <is>
           <t>lWC9k6Xq69PoP0M-UiJscZuSs-NM1jbc3aK2zyHKfIlTBpha1PE4Srp3CO7-jBLsWHXv4yuw--oUxQ</t>
@@ -20911,11 +20631,6 @@
           <t>uscs_hawks</t>
         </is>
       </c>
-      <c r="G695" t="inlineStr">
-        <is>
-          <t>uscs_hawks</t>
-        </is>
-      </c>
       <c r="I695" t="inlineStr">
         <is>
           <t>kwoCRlvJKOKZnqvre-rtLVpA9xF3DcIlvKs50HHUt7Ut1J7hItwYWqnybPUPzilSpis_Nxr9dCkWTQ</t>
@@ -21056,11 +20771,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G700" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I700" t="inlineStr">
         <is>
           <t>7d0hebUA4GEqkQxDBBhP5q6wnf3jc-i0KNTi4dnksWpl__ZIuySN0QwqeXifmsRE0Ygukj-evMkL7A</t>
@@ -21083,11 +20793,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G701" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="H701" t="inlineStr">
         <is>
           <t>macklogic_wine</t>
@@ -21439,11 +21144,6 @@
           <t>ufmt_turuna</t>
         </is>
       </c>
-      <c r="G714" t="inlineStr">
-        <is>
-          <t>ufmt_turuna</t>
-        </is>
-      </c>
       <c r="I714" t="inlineStr">
         <is>
           <t>0jpTPGN_JEwYgCuTUZsxHWHaLoDBphYgcttzYsfDyFGJzehatjfpv4qkrK11olQ7tYrSD2XC7A--yw</t>
@@ -22018,11 +21718,6 @@
           <t>ufscar_fire</t>
         </is>
       </c>
-      <c r="G736" t="inlineStr">
-        <is>
-          <t>ufscar_fire</t>
-        </is>
-      </c>
       <c r="I736" t="inlineStr">
         <is>
           <t>YxhqrMTfJPwiamZD6LzTGMMDngG9hg7P98PB6lsPgWQVf_XpDAucgXMkZvPFQXNOi9cKvru5Z_1XqA</t>
@@ -22099,11 +21794,6 @@
           <t>pucc_canaries</t>
         </is>
       </c>
-      <c r="G739" t="inlineStr">
-        <is>
-          <t>pucc_canaries</t>
-        </is>
-      </c>
       <c r="I739" t="inlineStr">
         <is>
           <t>Og1LoqH6b98DaYiu8Yb29wRQQOgAE7l1iS86k69tEH-pEPkIIIAJq3XA-ovATqLx394IczEvu-b6yw</t>
@@ -22122,11 +21812,6 @@
         </is>
       </c>
       <c r="B740" t="inlineStr">
-        <is>
-          <t>pucc_canaries</t>
-        </is>
-      </c>
-      <c r="G740" t="inlineStr">
         <is>
           <t>pucc_canaries</t>
         </is>

</xml_diff>

<commit_message>
checkpoint: trabalho local para continuar no Claude Cloud
Preserva o estado em andamento de cartinhas, comentarios, dados e ferramentas.
Inclui contexto de retomada e mantem originais de cartinhas futuras fora do repositorio publico.
O novo visual permanece na branch claude/visual-placar.
</commit_message>
<xml_diff>
--- a/dados_excel/players.xlsx
+++ b/dados_excel/players.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -941,11 +941,6 @@
           <t>wolf_gaming</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>wolf_gaming</t>
-        </is>
-      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>u9ICdhbvgpXi42XhszYP0F1LscHkpiee1a2DApmiP0OzsI98RdWD8mcygA1-IlPQIxVb8deraS_KXw</t>
@@ -1140,11 +1135,6 @@
           <t>usp_stars_gc</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>usp_stars_gc</t>
-        </is>
-      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>tAWTzpnPhLlsbGEYyNjIYcOm63rdaGGWGIMWrAvTCqSyR-ZI0gNvHsdH5fy37ddMcDIsPN0sZDnp6g</t>
@@ -1172,11 +1162,6 @@
           <t>usp_stars_gc</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>usp_stars_gc</t>
-        </is>
-      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>_WZpUmN7nBBFJ_MbGLditmDFthPf61fdPnYCei0g800r9lpc2My0rN31Dzoy4A_sbXIYGJ93wzSFMg</t>
@@ -1253,11 +1238,6 @@
           <t>usp_stars</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>usp_stars</t>
-        </is>
-      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>mEl8mUKuDxynBb38jXsHTBnE6F-z2OUzk8PKpKljnHcT1PRnkWKFM44I3ZxXLHUItzz6DOhi9ksSyA</t>
@@ -2309,11 +2289,6 @@
           <t>unirio_krakens</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>unirio_krakens</t>
-        </is>
-      </c>
       <c r="I64" t="inlineStr">
         <is>
           <t>Utp2yVXMV4mmUCo09_RcsF64VrOXnIqBtyA_-kE_UBXqKvib8yyFYMX8nAze_UKK4Z56ngWTSMe1NA</t>
@@ -3288,11 +3263,6 @@
           <t>unicamp_tritons_black</t>
         </is>
       </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>unicamp_tritons_black</t>
-        </is>
-      </c>
       <c r="I96" t="inlineStr">
         <is>
           <t>88G6xgaAAef5qemLkAbm_UEo1nWCPnK1V7WQBy49e1BS4cCCAVOi16Ml33pCXqu6FrPnfVZu6c--QA</t>
@@ -3903,11 +3873,6 @@
           <t>ufu_saints</t>
         </is>
       </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>ufu_saints</t>
-        </is>
-      </c>
       <c r="I116" t="inlineStr">
         <is>
           <t>PUcyfXweL2QkiapM6bxnyPCweB-ITtYFQHvdfkcSOPl1R0zdfUEgN7W0zs4M13zvj15XRUFd7W_GpQ</t>
@@ -3930,11 +3895,6 @@
           <t>ufu_saints</t>
         </is>
       </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>ufu_saints</t>
-        </is>
-      </c>
       <c r="I117" t="inlineStr">
         <is>
           <t>jfvKJJQmJ3vOg5rEUYN9Z67ibW2jnXGoQVITcE1IwK35-nsHLENNTnAN1npg0dzHUYERMrvzFbSM4A</t>
@@ -4058,11 +4018,6 @@
           <t>ufscar_fire</t>
         </is>
       </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>ufscar_fire</t>
-        </is>
-      </c>
       <c r="I121" t="inlineStr">
         <is>
           <t>bKsWXR9kAaZTMFmUA8Da_oBmzfFpE8JeS6QKFTUTmUprc8RSpLIw2FNBYRZNVpomvRshJzo1GI5S1g</t>
@@ -4626,11 +4581,6 @@
           <t>ufrj_minerva</t>
         </is>
       </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>ufrj_minerva</t>
-        </is>
-      </c>
       <c r="I140" t="inlineStr">
         <is>
           <t>im4BHDdELr1YKI4fX4mx9xS4hI-7SLWjsv8w16mAnyhyyylhbNh6jS_VtNuGIZjI-mZfZUddHWDLCA</t>
@@ -4948,11 +4898,6 @@
           <t>ufpr_bbn</t>
         </is>
       </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>ufpr_bbn</t>
-        </is>
-      </c>
       <c r="I151" t="inlineStr">
         <is>
           <t>bKYcnZJ-ToLmXHs45QuEJV7tdqCUIoMEU5-vFzBsAogC9VGqFN9puYwigg6JKcVd5caFm4145uN1lg</t>
@@ -4975,11 +4920,6 @@
           <t>ufpr_bbn</t>
         </is>
       </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>ufpr_bbn</t>
-        </is>
-      </c>
       <c r="I152" t="inlineStr">
         <is>
           <t>g-IvHtnI6kdiFnRFVnSVmtzKk8uZF4tulJpTcoqMe7tFgw5GXPJZ7xD7KxlfvqrJac5YHrRB7jYaTQ</t>
@@ -5179,11 +5119,6 @@
           <t>ufmt_turuna</t>
         </is>
       </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>ufmt_turuna</t>
-        </is>
-      </c>
       <c r="I159" t="inlineStr">
         <is>
           <t>WbmDscUxGUIMc2mq9e0W3SKTMxsMQL9xJ_P3jrFy4B5BATZ_9OaaUwDwznw2bFoBkZVnv6leOlzbpA</t>
@@ -6984,11 +6919,6 @@
           <t>totale_umc</t>
         </is>
       </c>
-      <c r="G224" t="inlineStr">
-        <is>
-          <t>totale_umc</t>
-        </is>
-      </c>
       <c r="I224" t="inlineStr">
         <is>
           <t>DEHyORp293uMthwlUKVrqEY7oQk3GK6YkM57y0eenYaqqZH4ZwBsRdZULpZth5GDPPB1s3kX6meaDQ</t>
@@ -7694,11 +7624,6 @@
           <t>pucgo_sistematica</t>
         </is>
       </c>
-      <c r="G249" t="inlineStr">
-        <is>
-          <t>pucgo_sistematica</t>
-        </is>
-      </c>
       <c r="I249" t="inlineStr">
         <is>
           <t>Plj4rlGsRBSkIKnfisJi-MV2sepg3SpaxRB98OoGga07acGP2eVLbgLqLIYxQjYeKc82FRlMFqkcrg</t>
@@ -7780,11 +7705,6 @@
           <t>pucgo_sistematica</t>
         </is>
       </c>
-      <c r="G252" t="inlineStr">
-        <is>
-          <t>pucgo_sistematica</t>
-        </is>
-      </c>
       <c r="I252" t="inlineStr">
         <is>
           <t>P8aY38Slk3RKg60vPOCKSsWTDmFKMsN6eTJjQLnUxvvwOgW33hejt3vmLnCKCncWxyoNmS7TO9i0gQ</t>
@@ -7834,11 +7754,6 @@
           <t>pucgo_sistematica</t>
         </is>
       </c>
-      <c r="G254" t="inlineStr">
-        <is>
-          <t>pucgo_sistematica</t>
-        </is>
-      </c>
       <c r="I254" t="inlineStr">
         <is>
           <t>dcX1EoCibLxmHNZRAyBwY-r81ItkAZe5NX2TtQXwbgY-YUdXSKSplOm7hL9pS-ftYB_ggFGkKY1Vhg</t>
@@ -7920,11 +7835,6 @@
           <t>pucc_cardinals</t>
         </is>
       </c>
-      <c r="G257" t="inlineStr">
-        <is>
-          <t>pucc_cardinals</t>
-        </is>
-      </c>
       <c r="I257" t="inlineStr">
         <is>
           <t>301qhx0vRdUVcofBGyq_VoAhuOwFm2GLKQ93asIyj37qjY-dG2lzyjNQHKIalkgRT4G9l7htJmVQkQ</t>
@@ -8053,11 +7963,6 @@
           <t>pucc_cardinals</t>
         </is>
       </c>
-      <c r="G261" t="inlineStr">
-        <is>
-          <t>pucc_cardinals</t>
-        </is>
-      </c>
       <c r="I261" t="inlineStr">
         <is>
           <t>ua9cSJ_WLHTDUhQhJYjkWcZ20qEiMBblpkY2SUuGfXrZij10AMpGNKivg1OCuCWXcJL5XN6ZNTcHcQ</t>
@@ -8080,11 +7985,6 @@
           <t>pucc_cardinals</t>
         </is>
       </c>
-      <c r="G262" t="inlineStr">
-        <is>
-          <t>pucc_cardinals</t>
-        </is>
-      </c>
       <c r="I262" t="inlineStr">
         <is>
           <t>QAn49vDOOkmlsACPBxsDlBH-p5bl93HPVr0DwAcwsPoqOEthQdSKL_2-ecm5IlT2uVxv52uuVrW4ew</t>
@@ -9437,11 +9337,6 @@
           <t>maua_blue</t>
         </is>
       </c>
-      <c r="G308" t="inlineStr">
-        <is>
-          <t>maua_blue</t>
-        </is>
-      </c>
       <c r="I308" t="inlineStr">
         <is>
           <t>HnS2m2EByAsSUFVsmd4FLWmlzRdtYLiURpHDpTYXYGZp6XS1YHKzXjPiBEe-biZAOcknSGbEcXyQ8w</t>
@@ -9464,11 +9359,6 @@
           <t>maua_blue</t>
         </is>
       </c>
-      <c r="G309" t="inlineStr">
-        <is>
-          <t>maua_blue</t>
-        </is>
-      </c>
       <c r="I309" t="inlineStr">
         <is>
           <t>5DtyRi2zT34YBGF66FSePkScbdKjEW9pPNB_aguFegUuHPK9kOvny5ZtfQfgzSYJgEEMjxDsiBMisA</t>
@@ -9518,11 +9408,6 @@
           <t>maua_blue</t>
         </is>
       </c>
-      <c r="G311" t="inlineStr">
-        <is>
-          <t>maua_blue</t>
-        </is>
-      </c>
       <c r="I311" t="inlineStr">
         <is>
           <t>gaSDlUryf--PXz557skg2GMkc2tLsessde_L76p-ArFgiId0mCbsPSnaDzS-mYuKT3MZiyBRNK_2Hg</t>
@@ -9577,11 +9462,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G313" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I313" t="inlineStr">
         <is>
           <t>2yslosTvB5-Q9mszSTYnUsHkt8dc2ryhnysRiaa_oUw7t3C45vaUQOWzro4OUYgztuiNKwu9zoaYtA</t>
@@ -9609,11 +9489,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G314" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I314" t="inlineStr">
         <is>
           <t>9edCRwvelp9Ko7rrbtTbk86da6un1VgQVZ7HFf0x3G8hmQbpGxGkY1D9QBQOYECuAHROjMACZxeW-g</t>
@@ -9636,11 +9511,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G315" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I315" t="inlineStr">
         <is>
           <t>DgRoFzXydtAKcOh2ntoyp6iqGyAOgMG3CWFcXnYTmmoGnijHaKCFS_u8tT47bILJOS8V_0mqSyVw2A</t>
@@ -9742,11 +9612,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G318" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I318" t="inlineStr">
         <is>
           <t>-SEFIRD9iWcerWPwSbl2xqpiq2BWZnWrBz8ZbT0Wl4-QpQ_LTtAxbBW_Y3qAdL9dr-EJPrQCQg5dtg</t>
@@ -9769,11 +9634,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G319" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I319" t="inlineStr">
         <is>
           <t>zUF3dytt7KB_gS05Zkpnmjb138wJb3onG45XJIDiMnS4m3NbY8dpaXSSfPCJGRvx0Gq4ZAOcliMayA</t>
@@ -9796,11 +9656,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G320" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="H320" t="inlineStr">
         <is>
           <t>macklogic_red; macklogic_wine</t>
@@ -9986,11 +9841,6 @@
           <t>macklogic_red</t>
         </is>
       </c>
-      <c r="G325" t="inlineStr">
-        <is>
-          <t>macklogic_red</t>
-        </is>
-      </c>
       <c r="I325" t="inlineStr">
         <is>
           <t>UMqsz421_7TZxaMOWSfkHTe8pC3sApewo-dX9I-Em4VbL0PwyTh6QNaYOT2chpOseS1UmfxTl9zkNQ</t>
@@ -10131,11 +9981,6 @@
           <t>macklogic_rainbow</t>
         </is>
       </c>
-      <c r="G330" t="inlineStr">
-        <is>
-          <t>macklogic_rainbow</t>
-        </is>
-      </c>
       <c r="I330" t="inlineStr">
         <is>
           <t>w8dgJVfD_Y64jJfKQRN8eKJNmxOeCnJEZnuGgJs5rlG3a_zdNycRrHlLyMw4ryNLeNoRai8a5jcA5A</t>
@@ -11057,11 +10902,6 @@
           <t>inatel_gray</t>
         </is>
       </c>
-      <c r="G363" t="inlineStr">
-        <is>
-          <t>inatel_gray</t>
-        </is>
-      </c>
       <c r="I363" t="inlineStr">
         <is>
           <t>PD2xOUFZLkq-i7-2FyDihzZEZNZtqNraY5XhJ0CqsB6WhXK9s-VtLuXy7dCepywKEjXgyyVPYp2Mvg</t>
@@ -11084,11 +10924,6 @@
           <t>inatel_gray</t>
         </is>
       </c>
-      <c r="G364" t="inlineStr">
-        <is>
-          <t>inatel_gray</t>
-        </is>
-      </c>
       <c r="I364" t="inlineStr">
         <is>
           <t>azLzX0-fc5yL96eqiV6QbzK6TmuOBf31YuoUScb0ELyWswIQDLOLoY5MbijUYfnGqUmJ-xqH_Odg-A</t>
@@ -12551,11 +12386,6 @@
           <t>green_owls_noctua</t>
         </is>
       </c>
-      <c r="G415" t="inlineStr">
-        <is>
-          <t>green_owls_noctua</t>
-        </is>
-      </c>
       <c r="I415" t="inlineStr">
         <is>
           <t>21R3F3xWR-kcyY9bP3cg684JI--MG0f3wv3loFoQPtR19ojbhniQ07Tr3yUusAi-ZoDgqs-rCMlR4Q</t>
@@ -12880,11 +12710,6 @@
           <t>gambiarra_ufg</t>
         </is>
       </c>
-      <c r="G427" t="inlineStr">
-        <is>
-          <t>gambiarra_ufg</t>
-        </is>
-      </c>
       <c r="L427" t="inlineStr">
         <is>
           <t>Thorfinn メ#naves</t>
@@ -12983,11 +12808,6 @@
           <t>furia_utfpr</t>
         </is>
       </c>
-      <c r="G431" t="inlineStr">
-        <is>
-          <t>furia_utfpr</t>
-        </is>
-      </c>
       <c r="I431" t="inlineStr">
         <is>
           <t>gfM9fyh51WHYAr4dX7Rnds0UKwEY3WfPFsncjdfcxYTE9s2NbsmzxurTn76dKcuXhwygOj3WR_EKjA</t>
@@ -14012,11 +13832,6 @@
           <t>ceub_octopus_vulgaris</t>
         </is>
       </c>
-      <c r="G463" t="inlineStr">
-        <is>
-          <t>ceub_octopus_vulgaris</t>
-        </is>
-      </c>
       <c r="H463" t="inlineStr">
         <is>
           <t>atletica_sustenta</t>
@@ -14801,11 +14616,6 @@
           <t>caap_malditos</t>
         </is>
       </c>
-      <c r="G485" t="inlineStr">
-        <is>
-          <t>caap_malditos</t>
-        </is>
-      </c>
       <c r="I485" t="inlineStr">
         <is>
           <t>E3ivYGaicB2XlnMhnolVgM0wf7s-1z7f3Xq8YCQtFgMsBw-I8ZFrfKmDgEeh7kD_k7P_AdfFuR20kg</t>
@@ -14966,11 +14776,6 @@
           <t>caap_hellhounds</t>
         </is>
       </c>
-      <c r="G490" t="inlineStr">
-        <is>
-          <t>caap_hellhounds</t>
-        </is>
-      </c>
       <c r="I490" t="inlineStr">
         <is>
           <t>_IMaT7l5138--TeO3kpZ_7ejIV_w32dNUnEmeJKzvNzh5KmslemzFZTQbydqibFW5ZHhifd-lcz54A</t>
@@ -15089,11 +14894,6 @@
           <t>caap_hellhounds</t>
         </is>
       </c>
-      <c r="G494" t="inlineStr">
-        <is>
-          <t>caap_hellhounds</t>
-        </is>
-      </c>
       <c r="I494" t="inlineStr">
         <is>
           <t>s_smSLBfGMdCnHDxwP0T0RFjRniaOr__qw72D73JzF7p4GXYPQx2qwbD2ILlrDsXPipLSplt3taL5Q</t>
@@ -15116,11 +14916,6 @@
           <t>caap_hellhounds</t>
         </is>
       </c>
-      <c r="G495" t="inlineStr">
-        <is>
-          <t>caap_hellhounds</t>
-        </is>
-      </c>
       <c r="I495" t="inlineStr">
         <is>
           <t>-k4zx9RhoxLQNGaEEVA4rw9o9_0HC-orLXCLIUtxJ0y8_-thVKLDNhfT1Ea-AGnXsOa0Nd0shSioYg</t>
@@ -15143,11 +14938,6 @@
           <t>caap_auroras</t>
         </is>
       </c>
-      <c r="G496" t="inlineStr">
-        <is>
-          <t>caap_auroras</t>
-        </is>
-      </c>
       <c r="I496" t="inlineStr">
         <is>
           <t>9gI-LexrKcJkxI1-xWQqbRSN8SwVvz3lwY3h0xBip886cf5g8L0sVQ9NogF70PfYCgb2VUy9HMJXsg</t>
@@ -15271,11 +15061,6 @@
           <t>caap_auroras</t>
         </is>
       </c>
-      <c r="G500" t="inlineStr">
-        <is>
-          <t>caap_auroras</t>
-        </is>
-      </c>
       <c r="I500" t="inlineStr">
         <is>
           <t>6jBTCJWXhj2d2kq6cTNjE3ykg55HXWJn0BHp59Yb_ukHkkflQn8JYca_mmFdESMmZI3jW94mEOdU8Q</t>
@@ -15753,11 +15538,6 @@
           <t>azure_bears_silver</t>
         </is>
       </c>
-      <c r="G516" t="inlineStr">
-        <is>
-          <t>azure_bears_silver</t>
-        </is>
-      </c>
       <c r="I516" t="inlineStr">
         <is>
           <t>FrflKIANQmKRQQTQPKmX0f8ZGnmo9n5eF42hWEDFL36laJkn_XbZX-u7VcHHNuOvsqMSgiKUc4zi9w</t>
@@ -15962,11 +15742,6 @@
           <t>azure_bears_golden</t>
         </is>
       </c>
-      <c r="G523" t="inlineStr">
-        <is>
-          <t>azure_bears_golden</t>
-        </is>
-      </c>
       <c r="I523" t="inlineStr">
         <is>
           <t>X6dK2xFXw4_isMR03zbzKl6bGGWP9X1kAFqdhsD4MV5qEcjArJhxIEiOp3xZP9fDpEUyCjNWTe2ajw</t>
@@ -16221,11 +15996,6 @@
           <t>azure_bears_black</t>
         </is>
       </c>
-      <c r="G530" t="inlineStr">
-        <is>
-          <t>azure_bears_black</t>
-        </is>
-      </c>
       <c r="I530" t="inlineStr">
         <is>
           <t>LBnUfrUKZa1Ry2fK1bWp7Ok0EizDW86Jd0jyt3FJJl044o3eS_2ZFcEICcjImD_Ow26oiKVSgFFvRg</t>
@@ -16610,11 +16380,6 @@
           <t>axis_anteaters</t>
         </is>
       </c>
-      <c r="G542" t="inlineStr">
-        <is>
-          <t>axis_anteaters</t>
-        </is>
-      </c>
       <c r="H542" t="inlineStr">
         <is>
           <t>sixa_eaters</t>
@@ -17445,11 +17210,6 @@
           <t>a2e_uff</t>
         </is>
       </c>
-      <c r="G567" t="inlineStr">
-        <is>
-          <t>a2e_uff</t>
-        </is>
-      </c>
       <c r="I567" t="inlineStr">
         <is>
           <t>YxfNWtbF20Z1tRTaFBSFyL1tHiLxkIV836jBLC96PNLp2lcAK-ZVauekN83dxgTq83Wdt6mwE4xUnQ</t>
@@ -17948,7 +17708,7 @@
     <row r="585">
       <c r="A585" t="inlineStr">
         <is>
-          <t>jotave</t>
+          <t>JotaVe</t>
         </is>
       </c>
       <c r="B585" t="inlineStr">
@@ -17963,7 +17723,7 @@
       </c>
       <c r="G585" t="inlineStr">
         <is>
-          <t>ceub_octopus_vulgaris</t>
+          <t>ceub_octopus</t>
         </is>
       </c>
       <c r="I585" t="inlineStr">
@@ -18121,11 +17881,6 @@
           <t>ceub_octopus_vulgaris</t>
         </is>
       </c>
-      <c r="G590" t="inlineStr">
-        <is>
-          <t>ceub_octopus_vulgaris</t>
-        </is>
-      </c>
       <c r="H590" t="inlineStr">
         <is>
           <t>atletica_sustenta</t>
@@ -18621,11 +18376,6 @@
           <t>ufu_saints</t>
         </is>
       </c>
-      <c r="G610" t="inlineStr">
-        <is>
-          <t>ufu_saints</t>
-        </is>
-      </c>
       <c r="I610" t="inlineStr">
         <is>
           <t>kVLPGLd0abwlSX6VkHzmWiuJtUe20TCvMaGG4R9bT6SezSyfhLjdcYO3gwzFMQciHDqNwOzQcfYkFg</t>
@@ -19499,11 +19249,6 @@
           <t>ufrj_minerva</t>
         </is>
       </c>
-      <c r="G644" t="inlineStr">
-        <is>
-          <t>ufrj_minerva</t>
-        </is>
-      </c>
       <c r="I644" t="inlineStr">
         <is>
           <t>6VmRqgEcADA3-FPKNyHudktkAmRCQ24f4-7qULqSetlt4BwhJOMPordrLxy5QW_H7xCbO87n8YDM4w</t>
@@ -19585,11 +19330,6 @@
           <t>ufrj_minerva</t>
         </is>
       </c>
-      <c r="G647" t="inlineStr">
-        <is>
-          <t>ufrj_minerva</t>
-        </is>
-      </c>
       <c r="I647" t="inlineStr">
         <is>
           <t>APM9XNdFLPZ0XIsxhQtKwlURG6MwycOF4EA0OZgJy-DCHEHh4vZmPDsjOjw2mUkEsJ-73BZEbseMrQ</t>
@@ -19774,11 +19514,6 @@
           <t>a2e_uff_shadows</t>
         </is>
       </c>
-      <c r="G654" t="inlineStr">
-        <is>
-          <t>a2e_uff_shadows</t>
-        </is>
-      </c>
       <c r="I654" t="inlineStr">
         <is>
           <t>K2nP5lhGeWcXKEoVzO1O-lICjLS4f2l_7X5U2uamQbAIxx3Jgkj_95sVV_ip-8TjWGrzQ1Yo4E049w</t>
@@ -19806,11 +19541,6 @@
           <t>a2e_uff</t>
         </is>
       </c>
-      <c r="G655" t="inlineStr">
-        <is>
-          <t>a2e_uff</t>
-        </is>
-      </c>
       <c r="I655" t="inlineStr">
         <is>
           <t>RRuFlSaUvwSAbsU0VZWUccWHztIDpZw_Q0uTHOpnzEfsCQUfxdzlNn3j5BEPEcQHEgwmSnmSfIzK1w</t>
@@ -20668,11 +20398,6 @@
           <t>brutal_esports</t>
         </is>
       </c>
-      <c r="G686" t="inlineStr">
-        <is>
-          <t>brutal_esports</t>
-        </is>
-      </c>
       <c r="I686" t="inlineStr">
         <is>
           <t>7Kip5H0Ns-j3RgPJqPL2CnGrSlwFygVFu8vG8IdWfuOVimmXaM-_kRhNAeipehmkzovgQGE5L80Ksw</t>
@@ -20695,11 +20420,6 @@
           <t>liga_vulkanica</t>
         </is>
       </c>
-      <c r="G687" t="inlineStr">
-        <is>
-          <t>liga_vulkanica</t>
-        </is>
-      </c>
       <c r="I687" t="inlineStr">
         <is>
           <t>lWC9k6Xq69PoP0M-UiJscZuSs-NM1jbc3aK2zyHKfIlTBpha1PE4Srp3CO7-jBLsWHXv4yuw--oUxQ</t>
@@ -20911,11 +20631,6 @@
           <t>uscs_hawks</t>
         </is>
       </c>
-      <c r="G695" t="inlineStr">
-        <is>
-          <t>uscs_hawks</t>
-        </is>
-      </c>
       <c r="I695" t="inlineStr">
         <is>
           <t>kwoCRlvJKOKZnqvre-rtLVpA9xF3DcIlvKs50HHUt7Ut1J7hItwYWqnybPUPzilSpis_Nxr9dCkWTQ</t>
@@ -21056,11 +20771,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G700" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="I700" t="inlineStr">
         <is>
           <t>7d0hebUA4GEqkQxDBBhP5q6wnf3jc-i0KNTi4dnksWpl__ZIuySN0QwqeXifmsRE0Ygukj-evMkL7A</t>
@@ -21083,11 +20793,6 @@
           <t>macklogic_white</t>
         </is>
       </c>
-      <c r="G701" t="inlineStr">
-        <is>
-          <t>macklogic_white</t>
-        </is>
-      </c>
       <c r="H701" t="inlineStr">
         <is>
           <t>macklogic_wine</t>
@@ -21439,11 +21144,6 @@
           <t>ufmt_turuna</t>
         </is>
       </c>
-      <c r="G714" t="inlineStr">
-        <is>
-          <t>ufmt_turuna</t>
-        </is>
-      </c>
       <c r="I714" t="inlineStr">
         <is>
           <t>0jpTPGN_JEwYgCuTUZsxHWHaLoDBphYgcttzYsfDyFGJzehatjfpv4qkrK11olQ7tYrSD2XC7A--yw</t>
@@ -22018,11 +21718,6 @@
           <t>ufscar_fire</t>
         </is>
       </c>
-      <c r="G736" t="inlineStr">
-        <is>
-          <t>ufscar_fire</t>
-        </is>
-      </c>
       <c r="I736" t="inlineStr">
         <is>
           <t>YxhqrMTfJPwiamZD6LzTGMMDngG9hg7P98PB6lsPgWQVf_XpDAucgXMkZvPFQXNOi9cKvru5Z_1XqA</t>
@@ -22099,11 +21794,6 @@
           <t>pucc_canaries</t>
         </is>
       </c>
-      <c r="G739" t="inlineStr">
-        <is>
-          <t>pucc_canaries</t>
-        </is>
-      </c>
       <c r="I739" t="inlineStr">
         <is>
           <t>Og1LoqH6b98DaYiu8Yb29wRQQOgAE7l1iS86k69tEH-pEPkIIIAJq3XA-ovATqLx394IczEvu-b6yw</t>
@@ -22122,11 +21812,6 @@
         </is>
       </c>
       <c r="B740" t="inlineStr">
-        <is>
-          <t>pucc_canaries</t>
-        </is>
-      </c>
-      <c r="G740" t="inlineStr">
         <is>
           <t>pucc_canaries</t>
         </is>

</xml_diff>